<commit_message>
lunes primero de junio carga masiva modulo
</commit_message>
<xml_diff>
--- a/public/assets/templates/plantilla_antropometria_digisalud.xlsx
+++ b/public/assets/templates/plantilla_antropometria_digisalud.xlsx
@@ -5,23 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nogue\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\digisalud_ve\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD75131C-C48F-43EE-9BF9-B2D86F6EAD2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628A489F-411D-4218-8CEA-EEE77D46A5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="2" r:id="rId1"/>
-    <sheet name="Antropometria" sheetId="1" r:id="rId2"/>
+    <sheet name="Antropometria" sheetId="1" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>id_digisalud</t>
   </si>
@@ -51,30 +51,6 @@
   </si>
   <si>
     <t>circ_cefalica_cm</t>
-  </si>
-  <si>
-    <t>VEMARIA...20080101</t>
-  </si>
-  <si>
-    <t>Maria</t>
-  </si>
-  <si>
-    <t>Perez</t>
-  </si>
-  <si>
-    <t>Menor de 19, cintura opcional</t>
-  </si>
-  <si>
-    <t>VEMJOSE...19850101</t>
-  </si>
-  <si>
-    <t>Jose</t>
-  </si>
-  <si>
-    <t>Rodriguez</t>
-  </si>
-  <si>
-    <t>Adulto, cintura obligatoria</t>
   </si>
   <si>
     <t>Plantilla carga masiva de antropometria</t>
@@ -387,99 +363,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
-  <cols>
-    <col min="1" max="1" width="110" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="22.35" customHeight="1">
-      <c r="A1" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
@@ -524,58 +407,26 @@
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="4">
-        <v>52.4</v>
-      </c>
-      <c r="E2" s="4">
-        <v>158</v>
-      </c>
-      <c r="F2" s="5">
-        <v>46171</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="5"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="4">
-        <v>23</v>
-      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="4"/>
       <c r="J2" s="4"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="4">
-        <v>82</v>
-      </c>
-      <c r="E3" s="4">
-        <v>172</v>
-      </c>
-      <c r="F3" s="5">
-        <v>46171</v>
-      </c>
-      <c r="G3" s="4">
-        <v>94</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="3"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
     </row>
@@ -6587,4 +6438,97 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="1" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="22.35" customHeight="1">
+      <c r="A1" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>